<commit_message>
fix(ml): calibrate camera model, 3D pose extraction, and normative reference distributions
</commit_message>
<xml_diff>
--- a/oa-sentinel-api-main/oa-sentinel-api-main/OA_Sentinel_Patient_Records.xlsx
+++ b/oa-sentinel-api-main/oa-sentinel-api-main/OA_Sentinel_Patient_Records.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q11"/>
+  <dimension ref="A1:Q29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1105,6 +1105,1164 @@
         </is>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-09-27T21:20:08</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>6ab93603aabe515c9f1946fe</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>49</v>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
+      <c r="E12" t="n">
+        <v>172</v>
+      </c>
+      <c r="F12" t="n">
+        <v>70</v>
+      </c>
+      <c r="G12" t="n">
+        <v>2</v>
+      </c>
+      <c r="H12" t="n">
+        <v>71.02</v>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>LOW PROTOTYPE RISK</t>
+        </is>
+      </c>
+      <c r="J12" t="n">
+        <v>0</v>
+      </c>
+      <c r="K12" t="n">
+        <v>0</v>
+      </c>
+      <c r="L12" t="n">
+        <v>97.95999999999999</v>
+      </c>
+      <c r="M12" t="n">
+        <v>8.16</v>
+      </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>right knee ROM below healthy 5th percentile</t>
+        </is>
+      </c>
+      <c r="O12" t="n">
+        <v>88.08</v>
+      </c>
+      <c r="P12" t="n">
+        <v>96.37</v>
+      </c>
+      <c r="Q12" t="inlineStr">
+        <is>
+          <t>Normative biomechanical screening only; not a clinical OA diagnosis or calibrated OA probability.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-09-27T21:24:15</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>OA-2026-524</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>48</v>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="E13" t="n">
+        <v>168</v>
+      </c>
+      <c r="F13" t="n">
+        <v>74</v>
+      </c>
+      <c r="G13" t="n">
+        <v>1</v>
+      </c>
+      <c r="H13" t="n">
+        <v>71.02</v>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>LOW PROTOTYPE RISK</t>
+        </is>
+      </c>
+      <c r="J13" t="n">
+        <v>0</v>
+      </c>
+      <c r="K13" t="n">
+        <v>0</v>
+      </c>
+      <c r="L13" t="n">
+        <v>97.95999999999999</v>
+      </c>
+      <c r="M13" t="n">
+        <v>8.16</v>
+      </c>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>right knee ROM below healthy 5th percentile; left knee ROM below healthy 5th percentile</t>
+        </is>
+      </c>
+      <c r="O13" t="n">
+        <v>88.08</v>
+      </c>
+      <c r="P13" t="n">
+        <v>96.37</v>
+      </c>
+      <c r="Q13" t="inlineStr">
+        <is>
+          <t>Normative biomechanical screening only; not a clinical OA diagnosis or calibrated OA probability.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-09-27T21:24:45</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>OA-2026-524</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>48</v>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="E14" t="n">
+        <v>168</v>
+      </c>
+      <c r="F14" t="n">
+        <v>74</v>
+      </c>
+      <c r="G14" t="n">
+        <v>1</v>
+      </c>
+      <c r="H14" t="n">
+        <v>71.02</v>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>LOW PROTOTYPE RISK</t>
+        </is>
+      </c>
+      <c r="J14" t="n">
+        <v>0</v>
+      </c>
+      <c r="K14" t="n">
+        <v>0</v>
+      </c>
+      <c r="L14" t="n">
+        <v>97.95999999999999</v>
+      </c>
+      <c r="M14" t="n">
+        <v>8.16</v>
+      </c>
+      <c r="N14" t="inlineStr">
+        <is>
+          <t>trunk lean above healthy 95th percentile; cadence below healthy 5th percentile; right knee ROM below healthy 5th percentile</t>
+        </is>
+      </c>
+      <c r="O14" t="n">
+        <v>88.08</v>
+      </c>
+      <c r="P14" t="n">
+        <v>96.37</v>
+      </c>
+      <c r="Q14" t="inlineStr">
+        <is>
+          <t>Normative biomechanical screening only; not a clinical OA diagnosis or calibrated OA probability.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2026-09-27T21:25:26</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>OA-2026-524</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>48</v>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="E15" t="n">
+        <v>168</v>
+      </c>
+      <c r="F15" t="n">
+        <v>74</v>
+      </c>
+      <c r="G15" t="n">
+        <v>1</v>
+      </c>
+      <c r="H15" t="n">
+        <v>71.02</v>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>LOW PROTOTYPE RISK</t>
+        </is>
+      </c>
+      <c r="J15" t="n">
+        <v>0</v>
+      </c>
+      <c r="K15" t="n">
+        <v>0</v>
+      </c>
+      <c r="L15" t="n">
+        <v>97.95999999999999</v>
+      </c>
+      <c r="M15" t="n">
+        <v>8.16</v>
+      </c>
+      <c r="N15" t="inlineStr">
+        <is>
+          <t>right knee ROM above healthy 95th percentile; left knee ROM above healthy 95th percentile</t>
+        </is>
+      </c>
+      <c r="O15" t="n">
+        <v>88.08</v>
+      </c>
+      <c r="P15" t="n">
+        <v>96.37</v>
+      </c>
+      <c r="Q15" t="inlineStr">
+        <is>
+          <t>Normative biomechanical screening only; not a clinical OA diagnosis or calibrated OA probability.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-09-27T21:25:48</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>OA-2026-524</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>48</v>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="E16" t="n">
+        <v>168</v>
+      </c>
+      <c r="F16" t="n">
+        <v>74</v>
+      </c>
+      <c r="G16" t="n">
+        <v>1</v>
+      </c>
+      <c r="H16" t="n">
+        <v>71.02</v>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>LOW PROTOTYPE RISK</t>
+        </is>
+      </c>
+      <c r="J16" t="n">
+        <v>0</v>
+      </c>
+      <c r="K16" t="n">
+        <v>0</v>
+      </c>
+      <c r="L16" t="n">
+        <v>97.95999999999999</v>
+      </c>
+      <c r="M16" t="n">
+        <v>8.16</v>
+      </c>
+      <c r="N16" t="inlineStr">
+        <is>
+          <t>trunk lean above healthy 95th percentile</t>
+        </is>
+      </c>
+      <c r="O16" t="n">
+        <v>88.08</v>
+      </c>
+      <c r="P16" t="n">
+        <v>96.37</v>
+      </c>
+      <c r="Q16" t="inlineStr">
+        <is>
+          <t>Normative biomechanical screening only; not a clinical OA diagnosis or calibrated OA probability.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-09-27T21:30:49</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>TEST-01</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>39</v>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr"/>
+      <c r="F17" t="inlineStr"/>
+      <c r="G17" t="n">
+        <v>1</v>
+      </c>
+      <c r="H17" t="n">
+        <v>100</v>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>HIGH PROTOTYPE RISK</t>
+        </is>
+      </c>
+      <c r="J17" t="n">
+        <v>-0.087991</v>
+      </c>
+      <c r="K17" t="n">
+        <v>100</v>
+      </c>
+      <c r="L17" t="n">
+        <v>100</v>
+      </c>
+      <c r="M17" t="n">
+        <v>100</v>
+      </c>
+      <c r="N17" t="inlineStr">
+        <is>
+          <t>cadence below healthy 5th percentile; right knee ROM below healthy 5th percentile</t>
+        </is>
+      </c>
+      <c r="O17" t="n">
+        <v>88.08</v>
+      </c>
+      <c r="P17" t="n">
+        <v>96.37</v>
+      </c>
+      <c r="Q17" t="inlineStr">
+        <is>
+          <t>Normative biomechanical screening only; not a clinical OA diagnosis or calibrated OA probability.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2026-09-27T21:32:03</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>OA-2026-524</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>48</v>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="E18" t="n">
+        <v>168</v>
+      </c>
+      <c r="F18" t="n">
+        <v>74</v>
+      </c>
+      <c r="G18" t="n">
+        <v>1</v>
+      </c>
+      <c r="H18" t="n">
+        <v>100</v>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>HIGH PROTOTYPE RISK</t>
+        </is>
+      </c>
+      <c r="J18" t="n">
+        <v>-0.145847</v>
+      </c>
+      <c r="K18" t="n">
+        <v>100</v>
+      </c>
+      <c r="L18" t="n">
+        <v>100</v>
+      </c>
+      <c r="M18" t="n">
+        <v>100</v>
+      </c>
+      <c r="N18" t="inlineStr">
+        <is>
+          <t>trunk lean above healthy 95th percentile; right knee ROM above healthy 95th percentile; left knee ROM above healthy 95th percentile</t>
+        </is>
+      </c>
+      <c r="O18" t="n">
+        <v>88.08</v>
+      </c>
+      <c r="P18" t="n">
+        <v>96.37</v>
+      </c>
+      <c r="Q18" t="inlineStr">
+        <is>
+          <t>Normative biomechanical screening only; not a clinical OA diagnosis or calibrated OA probability.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2026-09-27T21:33:00</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>OA-2026-524</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>48</v>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="E19" t="n">
+        <v>168</v>
+      </c>
+      <c r="F19" t="n">
+        <v>74</v>
+      </c>
+      <c r="G19" t="n">
+        <v>1</v>
+      </c>
+      <c r="H19" t="n">
+        <v>100</v>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>HIGH PROTOTYPE RISK</t>
+        </is>
+      </c>
+      <c r="J19" t="n">
+        <v>-0.155712</v>
+      </c>
+      <c r="K19" t="n">
+        <v>100</v>
+      </c>
+      <c r="L19" t="n">
+        <v>100</v>
+      </c>
+      <c r="M19" t="n">
+        <v>100</v>
+      </c>
+      <c r="N19" t="inlineStr">
+        <is>
+          <t>trunk lean above healthy 95th percentile; cadence below healthy 5th percentile; right knee ROM above healthy 95th percentile</t>
+        </is>
+      </c>
+      <c r="O19" t="n">
+        <v>88.08</v>
+      </c>
+      <c r="P19" t="n">
+        <v>96.37</v>
+      </c>
+      <c r="Q19" t="inlineStr">
+        <is>
+          <t>Normative biomechanical screening only; not a clinical OA diagnosis or calibrated OA probability.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2026-09-27T21:56:49</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>PATIENT-WALK-TEST</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>28</v>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr"/>
+      <c r="F20" t="inlineStr"/>
+      <c r="G20" t="n">
+        <v>1</v>
+      </c>
+      <c r="H20" t="n">
+        <v>1.03</v>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>LOW PROTOTYPE RISK</t>
+        </is>
+      </c>
+      <c r="J20" t="n">
+        <v>0.163568</v>
+      </c>
+      <c r="K20" t="n">
+        <v>0</v>
+      </c>
+      <c r="L20" t="n">
+        <v>1.47</v>
+      </c>
+      <c r="M20" t="n">
+        <v>0</v>
+      </c>
+      <c r="N20" t="inlineStr">
+        <is>
+          <t>No major measured deviation from the reference range</t>
+        </is>
+      </c>
+      <c r="O20" t="n">
+        <v>88.37</v>
+      </c>
+      <c r="P20" t="n">
+        <v>93.34999999999999</v>
+      </c>
+      <c r="Q20" t="inlineStr">
+        <is>
+          <t>Normative biomechanical screening only; not a clinical OA diagnosis or calibrated OA probability.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2026-09-27T21:56:57</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>PATIENT-WALK-TEST</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>28</v>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr"/>
+      <c r="F21" t="inlineStr"/>
+      <c r="G21" t="n">
+        <v>1</v>
+      </c>
+      <c r="H21" t="n">
+        <v>1.03</v>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>LOW PROTOTYPE RISK</t>
+        </is>
+      </c>
+      <c r="J21" t="n">
+        <v>0.163568</v>
+      </c>
+      <c r="K21" t="n">
+        <v>0</v>
+      </c>
+      <c r="L21" t="n">
+        <v>1.47</v>
+      </c>
+      <c r="M21" t="n">
+        <v>0</v>
+      </c>
+      <c r="N21" t="inlineStr">
+        <is>
+          <t>No major measured deviation from the reference range</t>
+        </is>
+      </c>
+      <c r="O21" t="n">
+        <v>88.37</v>
+      </c>
+      <c r="P21" t="n">
+        <v>93.34999999999999</v>
+      </c>
+      <c r="Q21" t="inlineStr">
+        <is>
+          <t>Normative biomechanical screening only; not a clinical OA diagnosis or calibrated OA probability.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2026-09-27T21:59:21</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>OA-2026-524</t>
+        </is>
+      </c>
+      <c r="C22" t="n">
+        <v>48</v>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="E22" t="n">
+        <v>168</v>
+      </c>
+      <c r="F22" t="n">
+        <v>74</v>
+      </c>
+      <c r="G22" t="n">
+        <v>1</v>
+      </c>
+      <c r="H22" t="n">
+        <v>53.78</v>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>MODERATE PROTOTYPE RISK</t>
+        </is>
+      </c>
+      <c r="J22" t="n">
+        <v>0.058697</v>
+      </c>
+      <c r="K22" t="n">
+        <v>0</v>
+      </c>
+      <c r="L22" t="n">
+        <v>76.81999999999999</v>
+      </c>
+      <c r="M22" t="n">
+        <v>0</v>
+      </c>
+      <c r="N22" t="inlineStr">
+        <is>
+          <t>trunk lean above healthy 95th percentile</t>
+        </is>
+      </c>
+      <c r="O22" t="n">
+        <v>88.37</v>
+      </c>
+      <c r="P22" t="n">
+        <v>93.34999999999999</v>
+      </c>
+      <c r="Q22" t="inlineStr">
+        <is>
+          <t>Normative biomechanical screening only; not a clinical OA diagnosis or calibrated OA probability.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>2026-09-27T22:00:06</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>OA-2026-524</t>
+        </is>
+      </c>
+      <c r="C23" t="n">
+        <v>48</v>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="E23" t="n">
+        <v>168</v>
+      </c>
+      <c r="F23" t="n">
+        <v>74</v>
+      </c>
+      <c r="G23" t="n">
+        <v>1</v>
+      </c>
+      <c r="H23" t="n">
+        <v>49.77</v>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>MODERATE PROTOTYPE RISK</t>
+        </is>
+      </c>
+      <c r="J23" t="n">
+        <v>0.06993099999999999</v>
+      </c>
+      <c r="K23" t="n">
+        <v>0</v>
+      </c>
+      <c r="L23" t="n">
+        <v>71.09999999999999</v>
+      </c>
+      <c r="M23" t="n">
+        <v>0</v>
+      </c>
+      <c r="N23" t="inlineStr">
+        <is>
+          <t>No major measured deviation from the reference range</t>
+        </is>
+      </c>
+      <c r="O23" t="n">
+        <v>88.37</v>
+      </c>
+      <c r="P23" t="n">
+        <v>93.34999999999999</v>
+      </c>
+      <c r="Q23" t="inlineStr">
+        <is>
+          <t>Normative biomechanical screening only; not a clinical OA diagnosis or calibrated OA probability.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>2026-09-27T22:00:46</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>OA-2026-524</t>
+        </is>
+      </c>
+      <c r="C24" t="n">
+        <v>48</v>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="E24" t="n">
+        <v>168</v>
+      </c>
+      <c r="F24" t="n">
+        <v>74</v>
+      </c>
+      <c r="G24" t="n">
+        <v>1</v>
+      </c>
+      <c r="H24" t="n">
+        <v>56.55</v>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>MODERATE PROTOTYPE RISK</t>
+        </is>
+      </c>
+      <c r="J24" t="n">
+        <v>0.049874</v>
+      </c>
+      <c r="K24" t="n">
+        <v>0</v>
+      </c>
+      <c r="L24" t="n">
+        <v>80.79000000000001</v>
+      </c>
+      <c r="M24" t="n">
+        <v>0</v>
+      </c>
+      <c r="N24" t="inlineStr">
+        <is>
+          <t>trunk lean above healthy 95th percentile</t>
+        </is>
+      </c>
+      <c r="O24" t="n">
+        <v>88.37</v>
+      </c>
+      <c r="P24" t="n">
+        <v>93.34999999999999</v>
+      </c>
+      <c r="Q24" t="inlineStr">
+        <is>
+          <t>Normative biomechanical screening only; not a clinical OA diagnosis or calibrated OA probability.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>2026-09-27T22:01:52</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>OA-2026-524</t>
+        </is>
+      </c>
+      <c r="C25" t="n">
+        <v>48</v>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="E25" t="n">
+        <v>168</v>
+      </c>
+      <c r="F25" t="n">
+        <v>74</v>
+      </c>
+      <c r="G25" t="n">
+        <v>1</v>
+      </c>
+      <c r="H25" t="n">
+        <v>60.3</v>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>MODERATE PROTOTYPE RISK</t>
+        </is>
+      </c>
+      <c r="J25" t="n">
+        <v>0.03741</v>
+      </c>
+      <c r="K25" t="n">
+        <v>0</v>
+      </c>
+      <c r="L25" t="n">
+        <v>85.45</v>
+      </c>
+      <c r="M25" t="n">
+        <v>1.62</v>
+      </c>
+      <c r="N25" t="inlineStr">
+        <is>
+          <t>left knee ROM above healthy 95th percentile</t>
+        </is>
+      </c>
+      <c r="O25" t="n">
+        <v>88.37</v>
+      </c>
+      <c r="P25" t="n">
+        <v>93.34999999999999</v>
+      </c>
+      <c r="Q25" t="inlineStr">
+        <is>
+          <t>Normative biomechanical screening only; not a clinical OA diagnosis or calibrated OA probability.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>2026-09-27T22:02:22</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>OA-2026-524</t>
+        </is>
+      </c>
+      <c r="C26" t="n">
+        <v>48</v>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="E26" t="n">
+        <v>168</v>
+      </c>
+      <c r="F26" t="n">
+        <v>74</v>
+      </c>
+      <c r="G26" t="n">
+        <v>1</v>
+      </c>
+      <c r="H26" t="n">
+        <v>78.38</v>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>HIGH PROTOTYPE RISK</t>
+        </is>
+      </c>
+      <c r="J26" t="n">
+        <v>-0.011326</v>
+      </c>
+      <c r="K26" t="n">
+        <v>100</v>
+      </c>
+      <c r="L26" t="n">
+        <v>96.7</v>
+      </c>
+      <c r="M26" t="n">
+        <v>35.62</v>
+      </c>
+      <c r="N26" t="inlineStr">
+        <is>
+          <t>trunk lean above healthy 95th percentile; right knee ROM above healthy 95th percentile; left knee ROM above healthy 95th percentile</t>
+        </is>
+      </c>
+      <c r="O26" t="n">
+        <v>88.37</v>
+      </c>
+      <c r="P26" t="n">
+        <v>93.34999999999999</v>
+      </c>
+      <c r="Q26" t="inlineStr">
+        <is>
+          <t>Normative biomechanical screening only; not a clinical OA diagnosis or calibrated OA probability.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>2026-09-27T22:02:46</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>OA-2026-524</t>
+        </is>
+      </c>
+      <c r="C27" t="n">
+        <v>48</v>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="E27" t="n">
+        <v>168</v>
+      </c>
+      <c r="F27" t="n">
+        <v>74</v>
+      </c>
+      <c r="G27" t="n">
+        <v>1</v>
+      </c>
+      <c r="H27" t="n">
+        <v>81.76000000000001</v>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>HIGH PROTOTYPE RISK</t>
+        </is>
+      </c>
+      <c r="J27" t="n">
+        <v>-0.021039</v>
+      </c>
+      <c r="K27" t="n">
+        <v>100</v>
+      </c>
+      <c r="L27" t="n">
+        <v>97.64</v>
+      </c>
+      <c r="M27" t="n">
+        <v>44.72</v>
+      </c>
+      <c r="N27" t="inlineStr">
+        <is>
+          <t>trunk lean above healthy 95th percentile; right knee ROM above healthy 95th percentile; left knee ROM above healthy 95th percentile</t>
+        </is>
+      </c>
+      <c r="O27" t="n">
+        <v>88.37</v>
+      </c>
+      <c r="P27" t="n">
+        <v>93.34999999999999</v>
+      </c>
+      <c r="Q27" t="inlineStr">
+        <is>
+          <t>Normative biomechanical screening only; not a clinical OA diagnosis or calibrated OA probability.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>2026-09-27T22:03:06</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>6ab93603aabe515c9f1946fe</t>
+        </is>
+      </c>
+      <c r="C28" t="n">
+        <v>49</v>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
+      <c r="E28" t="n">
+        <v>172</v>
+      </c>
+      <c r="F28" t="n">
+        <v>70</v>
+      </c>
+      <c r="G28" t="n">
+        <v>3</v>
+      </c>
+      <c r="H28" t="n">
+        <v>73.45999999999999</v>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>MODERATE PROTOTYPE RISK</t>
+        </is>
+      </c>
+      <c r="J28" t="n">
+        <v>0.001682</v>
+      </c>
+      <c r="K28" t="n">
+        <v>66.67</v>
+      </c>
+      <c r="L28" t="n">
+        <v>94.67</v>
+      </c>
+      <c r="M28" t="n">
+        <v>23.95</v>
+      </c>
+      <c r="N28" t="inlineStr">
+        <is>
+          <t>right knee ROM above healthy 95th percentile; left knee ROM above healthy 95th percentile</t>
+        </is>
+      </c>
+      <c r="O28" t="n">
+        <v>88.37</v>
+      </c>
+      <c r="P28" t="n">
+        <v>93.34999999999999</v>
+      </c>
+      <c r="Q28" t="inlineStr">
+        <is>
+          <t>Normative biomechanical screening only; not a clinical OA diagnosis or calibrated OA probability.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>2026-09-27T22:03:27</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>6ab93603aabe515c9f1946fb</t>
+        </is>
+      </c>
+      <c r="C29" t="n">
+        <v>58</v>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
+      <c r="E29" t="n">
+        <v>168</v>
+      </c>
+      <c r="F29" t="n">
+        <v>74</v>
+      </c>
+      <c r="G29" t="n">
+        <v>3</v>
+      </c>
+      <c r="H29" t="n">
+        <v>73.45999999999999</v>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>MODERATE PROTOTYPE RISK</t>
+        </is>
+      </c>
+      <c r="J29" t="n">
+        <v>0.001682</v>
+      </c>
+      <c r="K29" t="n">
+        <v>66.67</v>
+      </c>
+      <c r="L29" t="n">
+        <v>94.67</v>
+      </c>
+      <c r="M29" t="n">
+        <v>23.95</v>
+      </c>
+      <c r="N29" t="inlineStr">
+        <is>
+          <t>right knee ROM above healthy 95th percentile; left knee ROM above healthy 95th percentile</t>
+        </is>
+      </c>
+      <c r="O29" t="n">
+        <v>88.37</v>
+      </c>
+      <c r="P29" t="n">
+        <v>93.34999999999999</v>
+      </c>
+      <c r="Q29" t="inlineStr">
+        <is>
+          <t>Normative biomechanical screening only; not a clinical OA diagnosis or calibrated OA probability.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>